<commit_message>
make bullet weights less exaggerated (80gr/30 bullets to 0.01 weight)
</commit_message>
<xml_diff>
--- a/changes/545-ammo-super.xlsx
+++ b/changes/545-ammo-super.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yifan\Documents\deadline-balancing\changes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AFC58F3-F8D4-4233-B03C-9EFF65720DA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9CEC011-75DD-4E63-AB0A-5E3113EA29EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2018,7 +2018,7 @@
         <v>0</v>
       </c>
       <c r="D7" s="7">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="E7" s="38">
         <v>1</v>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="AL7" s="21">
         <f>C7*Model!$B$24+D7*Model!$B$25+E7*Model!$B$26+F7*Model!$B$27+G7*Model!$B$28+H7*Model!$B$29+I7*Model!$B$30+J7*Model!$B$31+K7*Model!$B$32</f>
-        <v>-3.0750000000000002</v>
+        <v>-2.875</v>
       </c>
       <c r="AM7" s="21">
         <f>(Z7-Model!$B$5)*Model!$B$35</f>
@@ -2148,7 +2148,7 @@
       </c>
       <c r="AQ7" s="21">
         <f t="shared" si="1"/>
-        <v>0.82900000000001484</v>
+        <v>1.029000000000015</v>
       </c>
     </row>
     <row r="8" spans="1:43">
@@ -2306,7 +2306,7 @@
         <v>-1</v>
       </c>
       <c r="D9" s="7">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="E9" s="38">
         <v>2</v>
@@ -2416,7 +2416,7 @@
       </c>
       <c r="AL9" s="21">
         <f>C9*Model!$B$24+D9*Model!$B$25+E9*Model!$B$26+F9*Model!$B$27+G9*Model!$B$28+H9*Model!$B$29+I9*Model!$B$30+J9*Model!$B$31+K9*Model!$B$32</f>
-        <v>-2.5</v>
+        <v>-2.3000000000000003</v>
       </c>
       <c r="AM9" s="21">
         <f>(Z9-Model!$B$5)*Model!$B$35</f>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="AQ9" s="21">
         <f t="shared" si="1"/>
-        <v>1.5406666666666666</v>
+        <v>1.7406666666666659</v>
       </c>
     </row>
     <row r="10" spans="1:43">
@@ -2450,7 +2450,7 @@
         <v>-1</v>
       </c>
       <c r="D10" s="7">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E10" s="38">
         <v>2</v>
@@ -2560,7 +2560,7 @@
       </c>
       <c r="AL10" s="21">
         <f>C10*Model!$B$24+D10*Model!$B$25+E10*Model!$B$26+F10*Model!$B$27+G10*Model!$B$28+H10*Model!$B$29+I10*Model!$B$30+J10*Model!$B$31+K10*Model!$B$32</f>
-        <v>-4</v>
+        <v>-3.6000000000000005</v>
       </c>
       <c r="AM10" s="21">
         <f>(Z10-Model!$B$5)*Model!$B$35</f>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="AQ10" s="21">
         <f t="shared" si="1"/>
-        <v>2.0106666666666682</v>
+        <v>2.4106666666666676</v>
       </c>
     </row>
     <row r="11" spans="1:43">
@@ -2594,7 +2594,7 @@
         <v>-1</v>
       </c>
       <c r="D11" s="7">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="E11" s="38">
         <v>2</v>
@@ -2704,7 +2704,7 @@
       </c>
       <c r="AL11" s="21">
         <f>C11*Model!$B$24+D11*Model!$B$25+E11*Model!$B$26+F11*Model!$B$27+G11*Model!$B$28+H11*Model!$B$29+I11*Model!$B$30+J11*Model!$B$31+K11*Model!$B$32</f>
-        <v>-3.3000000000000003</v>
+        <v>-2.9000000000000004</v>
       </c>
       <c r="AM11" s="21">
         <f>(Z11-Model!$B$5)*Model!$B$35</f>
@@ -2724,7 +2724,7 @@
       </c>
       <c r="AQ11" s="21">
         <f t="shared" si="1"/>
-        <v>1.8256666666666761</v>
+        <v>2.225666666666676</v>
       </c>
     </row>
     <row r="12" spans="1:43">
@@ -2738,7 +2738,7 @@
         <v>3</v>
       </c>
       <c r="D12" s="8">
-        <v>0.12</v>
+        <v>0.1</v>
       </c>
       <c r="E12" s="39">
         <v>-2</v>
@@ -2850,7 +2850,7 @@
       </c>
       <c r="AL12" s="22">
         <f>C12*Model!$B$24+D12*Model!$B$25+E12*Model!$B$26+F12*Model!$B$27+G12*Model!$B$28+H12*Model!$B$29+I12*Model!$B$30+J12*Model!$B$31+K12*Model!$B$32</f>
-        <v>-4.7</v>
+        <v>-4.3</v>
       </c>
       <c r="AM12" s="22">
         <f>(Z12-Model!$B$5)*Model!$B$35</f>
@@ -2870,7 +2870,7 @@
       </c>
       <c r="AQ12" s="22">
         <f t="shared" si="1"/>
-        <v>-5.2676666666666625</v>
+        <v>-4.8676666666666621</v>
       </c>
     </row>
   </sheetData>

</xml_diff>